<commit_message>
se actualiza el docstring de cada funcion
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
@@ -1862,10 +1862,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>44.35</v>
+        <v>42.92</v>
       </c>
       <c r="K12" t="n">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -2656,7 +2656,7 @@
         <v>99</v>
       </c>
       <c r="D12" t="n">
-        <v>8254</v>
+        <v>8257</v>
       </c>
       <c r="E12" t="n">
         <v>48.48</v>
@@ -3274,13 +3274,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D12" t="n">
-        <v>44.35</v>
+        <v>42.92</v>
       </c>
       <c r="E12" t="n">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3304,7 +3304,7 @@
         <v>32</v>
       </c>
       <c r="K12" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
-se generaron los datos de la hoja de resultados el excel resultante que compara el uso de cpu y memoria de las proyectos
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Errores" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Concurrencia" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Tokens" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Graficos" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="CPU-Memoria PC" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Graficos" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00\%"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -61,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -69,6 +72,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2073,7 +2079,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.01</v>
+        <v>2.94</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2081,7 +2087,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>46.99</v>
+        <v>45.64</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -2089,14 +2095,14 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>58.79</v>
+        <v>54.82</v>
       </c>
       <c r="K12" t="n">
-        <v>1.51</v>
+        <v>1.44</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Predominan issues medios</t>
+          <t>Predominan issues bajos</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -2497,16 +2503,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="C12" t="n">
-        <v>361</v>
+        <v>453</v>
       </c>
       <c r="D12" t="n">
-        <v>3.01</v>
+        <v>2.94</v>
       </c>
       <c r="E12" t="n">
-        <v>1616</v>
+        <v>1879</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -2519,7 +2525,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>13.47</v>
+        <v>12.2</v>
       </c>
     </row>
   </sheetData>
@@ -2879,16 +2885,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1616</v>
+        <v>1879</v>
       </c>
       <c r="C12" t="n">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="D12" t="n">
-        <v>9795</v>
+        <v>12139</v>
       </c>
       <c r="E12" t="n">
-        <v>46.99</v>
+        <v>45.64</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3503,41 +3509,41 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D12" t="n">
-        <v>58.79</v>
+        <v>54.82</v>
       </c>
       <c r="E12" t="n">
-        <v>1.51</v>
+        <v>1.44</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Predominan issues medios</t>
+          <t>Predominan issues bajos</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Contiene issues altos</t>
+          <t>Contiene issues medios</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="K12" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>mixed-line-endings: 23; broad-exception-caught: 10; trailing-whitespace: 10; 6/5: 8; 109/100: 4; subprocess-run-check: 4; 7/5: 4; 103/100: 3; no-value-for-parameter: 3; ungrouped-imports: 2</t>
+          <t>missing-function-docstring: 13; broad-exception-caught: 11; trailing-whitespace: 11; 6/5: 8; 109/100: 4; subprocess-run-check: 4; 103/100: 3; mixed-line-endings: 3; ungrouped-imports: 2; 101/100: 2</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3624,24 +3630,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Análisis concurrencia: No se encontró el código 'Propio' en Concurrencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Analizador metricas</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Análisis tokens: No se encontró el código 'Propio' en Datos Tokens</t>
+          <t>Análisis CPU/memoria: No se encontró el código 'Propio' en CPU_Memoria</t>
         </is>
       </c>
     </row>
@@ -4536,6 +4525,961 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:W12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="35" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="26" customWidth="1" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Lenguaje</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Método medición</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Modo CPU</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>CPUs lógicas</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Acción 1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>CPU medida 1</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Acción 2</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>CPU medida 2</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CPU normalizada 1</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>CPU normalizada 2</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>CPU promedio normalizada</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>CPU máxima normalizada</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Nivel CPU</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Interpretación CPU</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Memoria Acc1 (MB)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Memoria Acc2 (MB)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Memoria de total (MB)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Memoria promedio (MB)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Memoria normalizada promedio (%)</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Memoria máxima (MB)</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Nivel memoria</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Interpretación memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ps</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="Q2" s="4" t="n"/>
+      <c r="R2" s="4" t="n">
+        <v>4096</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="T2" s="5" t="n">
+        <v>0.0126953125</v>
+      </c>
+      <c r="U2" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>psutil</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="Q3" s="4" t="n"/>
+      <c r="R3" s="4" t="n">
+        <v>4096</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="T3" s="5" t="n">
+        <v>0.0166015625</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>M3-CC-Haiku</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ps</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>238</v>
+      </c>
+      <c r="Q4" s="4" t="n"/>
+      <c r="R4" s="4" t="n">
+        <v>8192</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>238</v>
+      </c>
+      <c r="T4" s="5" t="n">
+        <v>0.029052734375</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>238</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>M3-CC-Opus</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ps</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>8</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>238</v>
+      </c>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="n">
+        <v>8192</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>238</v>
+      </c>
+      <c r="T5" s="5" t="n">
+        <v>0.029052734375</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <v>238</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>M4-IDE-Gemini</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>psutil</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n">
+        <v>4096</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="T6" s="5" t="n">
+        <v>0.0048828125</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>M4-IDE-Sonnet</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>psutil</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q7" s="4" t="n"/>
+      <c r="R7" s="4" t="n">
+        <v>4096</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="T7" s="5" t="n">
+        <v>0.003662109375</v>
+      </c>
+      <c r="U7" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>M4-IDE-GPT</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>psutil</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" s="3" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n">
+        <v>2.6525</v>
+      </c>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n">
+        <v>2.6525</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>2.6525</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q8" s="4" t="n"/>
+      <c r="R8" s="4" t="n">
+        <v>4096</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="T8" s="5" t="n">
+        <v>0.0048828125</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>M4-IDE-Deepseek</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>psutil</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" s="3" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n">
+        <v>1.55375</v>
+      </c>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n">
+        <v>1.55375</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>1.55375</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q9" s="4" t="n"/>
+      <c r="R9" s="4" t="n">
+        <v>4096</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="T9" s="5" t="n">
+        <v>0.0048828125</v>
+      </c>
+      <c r="U9" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ps + jcmd</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" s="3" t="n">
+        <v>203.33</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n">
+        <v>25.41625</v>
+      </c>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n">
+        <v>25.41625</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>25.41625</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Consumo medio de CPU</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="Q10" s="4" t="n"/>
+      <c r="R10" s="4" t="n">
+        <v>8192</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="T10" s="5" t="n">
+        <v>0.0244140625</v>
+      </c>
+      <c r="U10" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>psutil</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>100%=1 núcleo</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" s="3" t="n">
+        <v>304</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Consumo medio de CPU</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>396</v>
+      </c>
+      <c r="Q11" s="4" t="n"/>
+      <c r="R11" s="4" t="n">
+        <v>16384</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>396</v>
+      </c>
+      <c r="T11" s="5" t="n">
+        <v>0.024169921875</v>
+      </c>
+      <c r="U11" s="4" t="n">
+        <v>396</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Propio</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" s="4" t="inlineStr"/>
+      <c r="Q12" s="4" t="inlineStr"/>
+      <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr"/>
+      <c r="T12" s="5" t="inlineStr"/>
+      <c r="U12" s="4" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData/>

</xml_diff>

<commit_message>
se dividio los umbrales de configuracion de cpu y memoria
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>45.64</v>
+        <v>45.67</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -2095,14 +2095,14 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>54.82</v>
+        <v>58.29</v>
       </c>
       <c r="K12" t="n">
-        <v>1.44</v>
+        <v>1.56</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Predominan issues bajos</t>
+          <t>Predominan issues medios</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
         <v>2.94</v>
       </c>
       <c r="E12" t="n">
-        <v>1879</v>
+        <v>1870</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -2525,7 +2525,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>12.2</v>
+        <v>12.14</v>
       </c>
     </row>
   </sheetData>
@@ -2885,16 +2885,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1879</v>
+        <v>1870</v>
       </c>
       <c r="C12" t="n">
         <v>154</v>
       </c>
       <c r="D12" t="n">
-        <v>12139</v>
+        <v>12161</v>
       </c>
       <c r="E12" t="n">
-        <v>45.64</v>
+        <v>45.67</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3509,41 +3509,41 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D12" t="n">
-        <v>54.82</v>
+        <v>58.29</v>
       </c>
       <c r="E12" t="n">
-        <v>1.44</v>
+        <v>1.56</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Moderada</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Predominan issues bajos</t>
+          <t>Predominan issues medios</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Contiene issues medios</t>
+          <t>Contiene issues altos</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J12" t="n">
         <v>45</v>
       </c>
       <c r="K12" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>missing-function-docstring: 13; broad-exception-caught: 11; trailing-whitespace: 11; 6/5: 8; 109/100: 4; subprocess-run-check: 4; 103/100: 3; mixed-line-endings: 3; ungrouped-imports: 2; 101/100: 2</t>
+          <t>missing-function-docstring: 13; trailing-whitespace: 12; broad-exception-caught: 11; 6/5: 8; 109/100: 4; subprocess-run-check: 4; 103/100: 3; 101/100: 3; no-value-for-parameter: 3; mixed-line-endings: 3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
se agregaron el uso de cpu y memoria en la hoja resumen
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
@@ -64,17 +64,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1249,7 +1248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1268,6 +1267,10 @@
     <col width="41" customWidth="1" min="14" max="14"/>
     <col width="27" customWidth="1" min="15" max="15"/>
     <col width="45" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="23" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="27" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1351,6 +1354,26 @@
           <t>Interpretación tokens</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>% CPU promedio</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Interpretación CPU</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>% Memoria promedio</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Interpretación memoria</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1421,6 +1444,22 @@
           <t>Alta NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="n">
+        <v>1.26953125</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1491,6 +1530,22 @@
           <t>Baja NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q3" s="2" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>1.66015625</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1561,6 +1616,22 @@
           <t>Baja NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q4" s="2" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>2.9052734375</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Consumo medio de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1631,6 +1702,22 @@
           <t>Baja NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q5" s="2" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>2.9052734375</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Consumo medio de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1701,6 +1788,22 @@
           <t>Alta NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q6" s="2" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0.48828125</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1771,6 +1874,22 @@
           <t>Alta NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q7" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>0.3662109375</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1841,6 +1960,22 @@
           <t>Alta NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q8" s="2" t="n">
+        <v>2.6525</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0.48828125</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1911,6 +2046,22 @@
           <t>Alta NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q9" s="2" t="n">
+        <v>1.55375</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Consumo bajo de CPU</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0.48828125</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Consumo bajo de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1981,6 +2132,22 @@
           <t>Baja NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q10" s="2" t="n">
+        <v>25.41625</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Consumo medio de CPU</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>2.44140625</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Consumo medio de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2051,6 +2218,22 @@
           <t>Alta NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
+      <c r="Q11" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Consumo medio de CPU</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>2.4169921875</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Consumo medio de memoria</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2079,7 +2262,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2.94</v>
+        <v>2.96</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2087,7 +2270,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>45.67</v>
+        <v>45.61</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -2095,10 +2278,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>58.29</v>
+        <v>59.26</v>
       </c>
       <c r="K12" t="n">
-        <v>1.56</v>
+        <v>1.54</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -2109,6 +2292,10 @@
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2503,16 +2690,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C12" t="n">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="D12" t="n">
-        <v>2.94</v>
+        <v>2.96</v>
       </c>
       <c r="E12" t="n">
-        <v>1870</v>
+        <v>1907</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -2525,7 +2712,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>12.14</v>
+        <v>12.3</v>
       </c>
     </row>
   </sheetData>
@@ -2885,16 +3072,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1870</v>
+        <v>1907</v>
       </c>
       <c r="C12" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D12" t="n">
-        <v>12161</v>
+        <v>12308</v>
       </c>
       <c r="E12" t="n">
-        <v>45.67</v>
+        <v>45.61</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3041,7 +3228,7 @@
       <c r="K2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>AvoidUsingVolatile: 2; ControlStatementBraces: 1; UseLocaleWithCaseConversions: 1</t>
         </is>
@@ -3091,7 +3278,7 @@
       <c r="K3" t="n">
         <v>70</v>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>missing-function-docstring: 40; import-error: 39; unused-variable: 13; logging-fstring-interpolation: 12; missing-module-docstring: 11; missing-class-docstring: 8; f-string-without-interpolation: 8; broad-exception-caught: 7; wrong-import-order: 7; global-statement: 3</t>
         </is>
@@ -3141,7 +3328,7 @@
       <c r="K4" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>GuardLogStatement: 22; CloseResource: 8; ControlStatementBraces: 4; LooseCoupling: 3; UseLocaleWithCaseConversions: 2; OneDeclarationPerLine: 1; UncommentedEmptyConstructor: 1</t>
         </is>
@@ -3191,7 +3378,7 @@
       <c r="K5" t="n">
         <v>5</v>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>ControlStatementBraces: 13; GuardLogStatement: 7; LooseCoupling: 5; CloseResource: 3; UselessParentheses: 3; OneDeclarationPerLine: 2; UncommentedEmptyConstructor: 1</t>
         </is>
@@ -3241,7 +3428,7 @@
       <c r="K6" t="n">
         <v>45</v>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>trailing-whitespace: 34; logging-fstring-interpolation: 10; invalid-name: 5; line 306: 4; 105/100: 1; 108/100: 1; 104/100: 1; 107/100: 1; missing-final-newline: 1; missing-module-docstring: 1</t>
         </is>
@@ -3291,7 +3478,7 @@
       <c r="K7" t="n">
         <v>5</v>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>logging-fstring-interpolation: 27; 6/5: 6; 7/5: 4; 10/7: 2; consider-using-max-builtin: 2; 111/100: 1; 123/100: 1; 115/100: 1; missing-class-docstring: 1; 9/7: 1</t>
         </is>
@@ -3341,7 +3528,7 @@
       <c r="K8" t="n">
         <v>28</v>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t>logging-fstring-interpolation: 5; broad-exception-caught: 4; 6/5: 4; 101/100: 3; 146/100: 2; 1/2: 2; 7/5: 2; 8/5: 2; 9/5: 2; unused-import: 2</t>
         </is>
@@ -3391,7 +3578,7 @@
       <c r="K9" t="n">
         <v>12</v>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>logging-fstring-interpolation: 21; missing-function-docstring: 5; broad-exception-caught: 4; 6/5: 4; 105/100: 1; 125/100: 1; 119/100: 1; 147/100: 1; 102/100: 1; missing-class-docstring: 1</t>
         </is>
@@ -3441,7 +3628,7 @@
       <c r="K10" t="n">
         <v>13</v>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t>PackageCase: 46; UnusedPrivateField: 38; ForLoopCanBeForeach: 25; LooseCoupling: 19; CloseResource: 10; UselessParentheses: 7; CompareObjectsWithEquals: 6; UnusedFormalParameter: 5; UnnecessaryFullyQualifiedName: 4; UncommentedEmptyMethodBody: 3</t>
         </is>
@@ -3491,7 +3678,7 @@
       <c r="K11" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t>import-error: 2; 1/2: 2; fixme: 1; 6/5: 1</t>
         </is>
@@ -3509,13 +3696,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D12" t="n">
-        <v>58.29</v>
+        <v>59.26</v>
       </c>
       <c r="E12" t="n">
-        <v>1.56</v>
+        <v>1.54</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3539,11 +3726,11 @@
         <v>45</v>
       </c>
       <c r="K12" t="n">
-        <v>60</v>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>missing-function-docstring: 13; trailing-whitespace: 12; broad-exception-caught: 11; 6/5: 8; 109/100: 4; subprocess-run-check: 4; 103/100: 3; 101/100: 3; no-value-for-parameter: 3; mixed-line-endings: 3</t>
+        <v>64</v>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>trailing-whitespace: 17; missing-function-docstring: 13; broad-exception-caught: 11; 6/5: 8; 109/100: 4; subprocess-run-check: 4; 8/5: 4; 103/100: 3; 101/100: 3; no-value-for-parameter: 3</t>
         </is>
       </c>
     </row>
@@ -3558,7 +3745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3629,6 +3816,57 @@
         </is>
       </c>
       <c r="C4" t="inlineStr">
+        <is>
+          <t>Análisis CPU/memoria: No se encontró el código 'Propio' en CPU_Memoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Propio</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Analizador metricas</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Análisis concurrencia: No se encontró el código 'Propio' en Concurrencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Propio</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Analizador metricas</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Análisis tokens: No se encontró el código 'Propio' en Datos Tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Propio</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Analizador metricas</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>Análisis CPU/memoria: No se encontró el código 'Propio' en CPU_Memoria</t>
         </is>
@@ -4550,7 +4788,7 @@
     <col width="35" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="26" customWidth="1" min="23" max="23"/>
+    <col width="27" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4695,19 +4933,19 @@
         <v>4</v>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="2" t="n">
         <v>4</v>
       </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n">
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n">
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="M2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N2" t="inlineStr">
@@ -4730,8 +4968,8 @@
       <c r="S2" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="T2" s="5" t="n">
-        <v>0.0126953125</v>
+      <c r="T2" s="2" t="n">
+        <v>1.26953125</v>
       </c>
       <c r="U2" s="4" t="n">
         <v>52</v>
@@ -4772,19 +5010,19 @@
         <v>8</v>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n">
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n">
         <v>6.25</v>
       </c>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n">
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n">
         <v>6.25</v>
       </c>
-      <c r="M3" s="3" t="n">
+      <c r="M3" s="2" t="n">
         <v>6.25</v>
       </c>
       <c r="N3" t="inlineStr">
@@ -4807,8 +5045,8 @@
       <c r="S3" s="4" t="n">
         <v>68</v>
       </c>
-      <c r="T3" s="5" t="n">
-        <v>0.0166015625</v>
+      <c r="T3" s="2" t="n">
+        <v>1.66015625</v>
       </c>
       <c r="U3" s="4" t="n">
         <v>68</v>
@@ -4849,19 +5087,19 @@
         <v>8</v>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="2" t="n">
         <v>42</v>
       </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n">
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n">
         <v>5.25</v>
       </c>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n">
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n">
         <v>5.25</v>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="M4" s="2" t="n">
         <v>5.25</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -4884,20 +5122,20 @@
       <c r="S4" s="4" t="n">
         <v>238</v>
       </c>
-      <c r="T4" s="5" t="n">
-        <v>0.029052734375</v>
+      <c r="T4" s="2" t="n">
+        <v>2.9052734375</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>238</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Medio</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo medio de memoria</t>
         </is>
       </c>
     </row>
@@ -4926,19 +5164,19 @@
         <v>8</v>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="2" t="n">
         <v>42</v>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n">
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n">
         <v>5.25</v>
       </c>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n">
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n">
         <v>5.25</v>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="M5" s="2" t="n">
         <v>5.25</v>
       </c>
       <c r="N5" t="inlineStr">
@@ -4961,20 +5199,20 @@
       <c r="S5" s="4" t="n">
         <v>238</v>
       </c>
-      <c r="T5" s="5" t="n">
-        <v>0.029052734375</v>
+      <c r="T5" s="2" t="n">
+        <v>2.9052734375</v>
       </c>
       <c r="U5" s="4" t="n">
         <v>238</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Medio</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo medio de memoria</t>
         </is>
       </c>
     </row>
@@ -5003,19 +5241,19 @@
         <v>4</v>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" s="3" t="n">
+      <c r="G6" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n">
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n">
         <v>0.125</v>
       </c>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n">
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n">
         <v>0.125</v>
       </c>
-      <c r="M6" s="3" t="n">
+      <c r="M6" s="2" t="n">
         <v>0.125</v>
       </c>
       <c r="N6" t="inlineStr">
@@ -5038,8 +5276,8 @@
       <c r="S6" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="T6" s="5" t="n">
-        <v>0.0048828125</v>
+      <c r="T6" s="2" t="n">
+        <v>0.48828125</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>20</v>
@@ -5080,19 +5318,19 @@
         <v>4</v>
       </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" s="3" t="n">
+      <c r="G7" s="2" t="n">
         <v>0.2</v>
       </c>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n">
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n">
         <v>0.05</v>
       </c>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n">
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n">
         <v>0.05</v>
       </c>
-      <c r="M7" s="3" t="n">
+      <c r="M7" s="2" t="n">
         <v>0.05</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -5115,8 +5353,8 @@
       <c r="S7" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="T7" s="5" t="n">
-        <v>0.003662109375</v>
+      <c r="T7" s="2" t="n">
+        <v>0.3662109375</v>
       </c>
       <c r="U7" s="4" t="n">
         <v>15</v>
@@ -5157,19 +5395,19 @@
         <v>4</v>
       </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" s="3" t="n">
+      <c r="G8" s="2" t="n">
         <v>10.61</v>
       </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n">
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n">
         <v>2.6525</v>
       </c>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n">
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n">
         <v>2.6525</v>
       </c>
-      <c r="M8" s="3" t="n">
+      <c r="M8" s="2" t="n">
         <v>2.6525</v>
       </c>
       <c r="N8" t="inlineStr">
@@ -5192,8 +5430,8 @@
       <c r="S8" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="T8" s="5" t="n">
-        <v>0.0048828125</v>
+      <c r="T8" s="2" t="n">
+        <v>0.48828125</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>20</v>
@@ -5234,19 +5472,19 @@
         <v>8</v>
       </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" s="3" t="n">
+      <c r="G9" s="2" t="n">
         <v>12.43</v>
       </c>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n">
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n">
         <v>1.55375</v>
       </c>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n">
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n">
         <v>1.55375</v>
       </c>
-      <c r="M9" s="3" t="n">
+      <c r="M9" s="2" t="n">
         <v>1.55375</v>
       </c>
       <c r="N9" t="inlineStr">
@@ -5269,8 +5507,8 @@
       <c r="S9" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="T9" s="5" t="n">
-        <v>0.0048828125</v>
+      <c r="T9" s="2" t="n">
+        <v>0.48828125</v>
       </c>
       <c r="U9" s="4" t="n">
         <v>20</v>
@@ -5311,19 +5549,19 @@
         <v>8</v>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" s="3" t="n">
+      <c r="G10" s="2" t="n">
         <v>203.33</v>
       </c>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n">
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n">
         <v>25.41625</v>
       </c>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n">
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n">
         <v>25.41625</v>
       </c>
-      <c r="M10" s="3" t="n">
+      <c r="M10" s="2" t="n">
         <v>25.41625</v>
       </c>
       <c r="N10" t="inlineStr">
@@ -5346,20 +5584,20 @@
       <c r="S10" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="T10" s="5" t="n">
-        <v>0.0244140625</v>
+      <c r="T10" s="2" t="n">
+        <v>2.44140625</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>200</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Medio</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo medio de memoria</t>
         </is>
       </c>
     </row>
@@ -5388,19 +5626,19 @@
         <v>8</v>
       </c>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" s="3" t="n">
+      <c r="G11" s="2" t="n">
         <v>304</v>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n">
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n">
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="M11" s="3" t="n">
+      <c r="M11" s="2" t="n">
         <v>38</v>
       </c>
       <c r="N11" t="inlineStr">
@@ -5423,20 +5661,20 @@
       <c r="S11" s="4" t="n">
         <v>396</v>
       </c>
-      <c r="T11" s="5" t="n">
-        <v>0.024169921875</v>
+      <c r="T11" s="2" t="n">
+        <v>2.4169921875</v>
       </c>
       <c r="U11" s="4" t="n">
         <v>396</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Medio</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo medio de memoria</t>
         </is>
       </c>
     </row>
@@ -5451,20 +5689,20 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" s="4" t="inlineStr"/>
       <c r="Q12" s="4" t="inlineStr"/>
       <c r="R12" s="4" t="inlineStr"/>
       <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="5" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="4" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>

</xml_diff>

<commit_message>
-se optimizo el codigo con constantes/definiciones.py
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
@@ -1270,7 +1270,7 @@
     <col width="17" customWidth="1" min="17" max="17"/>
     <col width="23" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
-    <col width="27" customWidth="1" min="20" max="20"/>
+    <col width="25" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Baja NLOC/token, ajustada por refinamientos.</t>
+          <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q3" s="2" t="n">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Baja NLOC/token, ajustada por refinamientos.</t>
+          <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q4" s="2" t="n">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Consumo medio de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Baja NLOC/token, ajustada por refinamientos.</t>
+          <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q5" s="2" t="n">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Consumo medio de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q6" s="2" t="n">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q7" s="2" t="n">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q8" s="2" t="n">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q9" s="2" t="n">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Baja NLOC/token, ajustada por refinamientos.</t>
+          <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q10" s="2" t="n">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Consumo medio de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -2215,7 +2215,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
       <c r="Q11" s="2" t="n">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Consumo medio de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2.96</v>
+        <v>2.86</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2270,7 +2270,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>45.61</v>
+        <v>45.92</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -2278,10 +2278,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>59.26</v>
+        <v>82.67</v>
       </c>
       <c r="K12" t="n">
-        <v>1.54</v>
+        <v>1.59</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -2690,16 +2690,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C12" t="n">
-        <v>459</v>
+        <v>441</v>
       </c>
       <c r="D12" t="n">
-        <v>2.96</v>
+        <v>2.86</v>
       </c>
       <c r="E12" t="n">
-        <v>1907</v>
+        <v>1875</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>12.3</v>
+        <v>12.18</v>
       </c>
     </row>
   </sheetData>
@@ -3072,16 +3072,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1907</v>
+        <v>1875</v>
       </c>
       <c r="C12" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D12" t="n">
-        <v>12308</v>
+        <v>12156</v>
       </c>
       <c r="E12" t="n">
-        <v>45.61</v>
+        <v>45.92</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3206,7 +3206,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Contiene issues altos</t>
+          <t>Contiene issues medios</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3366,7 +3366,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Contiene issues altos</t>
+          <t>Contiene issues medios</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Bajo</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3416,7 +3416,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Contiene issues medios</t>
+          <t>solo issues bajos</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Bajo</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3516,7 +3516,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Contiene issues medios</t>
+          <t>solo issues bajos</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Contiene issues altos</t>
+          <t>Contiene issues medios</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3696,17 +3696,17 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>113</v>
+        <v>155</v>
       </c>
       <c r="D12" t="n">
-        <v>59.26</v>
+        <v>82.67</v>
       </c>
       <c r="E12" t="n">
-        <v>1.54</v>
+        <v>1.59</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -3716,21 +3716,21 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Contiene issues altos</t>
+          <t>Contiene issues medios</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="J12" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="K12" t="n">
-        <v>64</v>
+        <v>97</v>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>trailing-whitespace: 17; missing-function-docstring: 13; broad-exception-caught: 11; 6/5: 8; 109/100: 4; subprocess-run-check: 4; 8/5: 4; 103/100: 3; 101/100: 3; no-value-for-parameter: 3</t>
+          <t>trailing-whitespace: 21; missing-function-docstring: 18; broad-exception-caught: 11; no-value-for-parameter: 9; 6/5: 8; 104/100: 7; 103/100: 5; subprocess-run-check: 4; unused-import: 4; 8/5: 4</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3816,57 +3816,6 @@
         </is>
       </c>
       <c r="C4" t="inlineStr">
-        <is>
-          <t>Análisis CPU/memoria: No se encontró el código 'Propio' en CPU_Memoria</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Analizador metricas</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Análisis concurrencia: No se encontró el código 'Propio' en Concurrencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Analizador metricas</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Análisis tokens: No se encontró el código 'Propio' en Datos Tokens</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Analizador metricas</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
         <is>
           <t>Análisis CPU/memoria: No se encontró el código 'Propio' en CPU_Memoria</t>
         </is>
@@ -4400,7 +4349,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4386,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Baja NLOC/token, ajustada por refinamientos.</t>
+          <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4474,7 +4423,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Baja NLOC/token, ajustada por refinamientos.</t>
+          <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4460,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Baja NLOC/token, ajustada por refinamientos.</t>
+          <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4497,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4534,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4622,7 +4571,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4659,7 +4608,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4696,7 +4645,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Baja NLOC/token, ajustada por refinamientos.</t>
+          <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4682,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Alta NLOC/token, ajustada por refinamientos.</t>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4737,7 @@
     <col width="35" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="27" customWidth="1" min="23" max="23"/>
+    <col width="25" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4981,7 +4930,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -5058,7 +5007,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -5130,12 +5079,12 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Bajo</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>Consumo medio de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -5207,12 +5156,12 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Bajo</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Consumo medio de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -5289,7 +5238,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5315,7 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -5443,7 +5392,7 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -5520,7 +5469,7 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Consumo bajo de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -5592,12 +5541,12 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Bajo</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>Consumo medio de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>
@@ -5669,12 +5618,12 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Bajo</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>Consumo medio de memoria</t>
+          <t>Consumo bajo de CPU</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
se crearon los graficos de uso de cpu y memoria
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_calidad_resultados.xlsx
@@ -822,6 +822,230 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>% Uso CPU</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Resumen'!Q1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Resumen'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumen'!$Q$2:$Q$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Proyecto</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Uso CPU</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>% Uso Memoria</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Resumen'!S1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Resumen'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumen'!$S$2:$S$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Proyecto</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Uso Memoria</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -951,6 +1175,50 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>113</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="7" name="Chart 7"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>132</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="8" name="Chart 8"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId8"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>